<commit_message>
Make instructions tab client-ready for segment leads
Tab renamed to 'How to read' and stripped to: how-to-read guidance,
aggregate priorities, and segment priorities. Removed the internal
Notes, Terminology and Open questions sections and all working-session
attributions. Milestones bullet reworded to 'major proposition-related
milestones over the horizon in which they land'. 'Corporate priorities
/ constraints' relabeled to 'Corporate priorities' across all tabs of
all three workbooks.

https://claude.ai/code/session_011p8iTtbymDUbCg8RtXLgqJ
</commit_message>
<xml_diff>
--- a/TAM2.0_Sequencing_Prework_Enterprise_v0.2.xlsx
+++ b/TAM2.0_Sequencing_Prework_Enterprise_v0.2.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Notes — READ ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How to read" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Global — cross-region" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Europe" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="APAC" sheetId="4" state="visible" r:id="rId4"/>
@@ -115,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -137,11 +137,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -188,6 +232,8 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -553,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A50"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="135" customWidth="1" min="1" max="1"/>
@@ -573,290 +619,132 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
+          <t>How to read this workbook:</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. Unlike the PPT exercise we did for Genius, this is a geo × segment view.</t>
+          <t>• Each geo tab opens with the inputs: business priorities and corporate priorities, with the dates by which they must be met.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2. It takes business priorities and corporate priorities as inputs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>• The Milestones row (▼) places major proposition-related milestones over the horizon in which they land.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>3. It captures the current-state and target-state stack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
+          <t>• Each workstream row shows the current-state stack, the target-state stack, and the planned actions across Now (H2 '26 – H1 '27), Next (H2 '27 – H1 '29) and Later (H2 '29+).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>4. It tracks BUILD, MIGRATE and DECOM decisions on a Now / Next / Later timeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>How to read each geo tab:</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
+          <t>• Actions are tagged: [BUILD] target-state build · [MIGRATE] migration or thin-out · [STOP] stop-sell / stop-integration · [EXIT] decommission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>• Square brackets denote channel context where relevant, e.g. [Bank], [ISV], [Payrix].</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>• Content is scoped to TAM 2.0 — platform-rationalisation actions, not the full BAU roadmap. Where an action enables a stated business priority, the cell says so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>• The INPUTS box holds business priorities and corporate constraints, with the dates they must be met. Segment-level priorities (below) sit above the geo-level priorities captured on each tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
+          <t>• Data centre consolidation is tracked under the Global Infrastructure &amp; Security workstream.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>• The Milestones row (▼) places proposition and corporate milestones over the horizon in which they land.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>• The table has one row per workstream: current-state stack, target-state stack, then Now / Next / Later actions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>• All timeline activities are TAM-scoped; BAU roadmap items are excluded. Where an activity directly enables a stated business priority, the cell says so: "[BUILD] … — enabling &lt;priority&gt;".</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
+          <t>• Blue text is a working hypothesis for validation. A blank cell is a request for input — not an indication that nothing is planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Aggregate priorities (segment-wide, 2026–27):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>• Tags: [BUILD] = target-state build or adherence · [MIGRATE] = front-book switch, back-book migration or thin-out · [STOP] = stop-sell / stop-integration (frees capacity) · [EXIT] = decommission milestone.</t>
+          <t>• Standardization and platform unification (POM + TAM).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>• Channel / persona context is tagged inline in square brackets where relevant, e.g. [Bank], [ISV], [Wholesale].</t>
+          <t>• Onboarding and activation speed — the core growth bottleneck.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>• Data centre consolidation is tracked under the Global Infrastructure &amp; Security workstream.</t>
+          <t>• VAS monetization — lending, payments optimization, settlement.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>• Horizons: Now = H2 '26 – H1 '27 · Next = H2 '27 – H1 '29 · Later = H2 '29+.</t>
+          <t>• Execution discipline — customer commitments and large rollouts.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>• Blue text is a hypothesis to validate. A blank cell means we need your input — not that nothing is planned.</t>
-        </is>
-      </c>
-    </row>
+          <t>• Migration off legacy and reduction of fragmentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Terminology:</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1">
+          <t>Enterprise segment priorities:</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>• Sales motion = direct, partner-led, or self-serve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
+          <t>• 2026 — Expand global payment capabilities (APMs, card acceptance, hosted payouts and in-app solutions). Enable complex enterprise use cases (marketplace and platform capabilities: split payments, cross-border collection, embedded payouts and treasury flows). Launch next-gen commerce (agentic commerce foundations; tokenized payments and AI integrations). Optimize partner and cost structure (third-party dependencies, partner agreements, commercial models).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>• Persona = the partner or customer type within a segment (e.g. Referral, Agent, ISO/Wholesale, Payfac, PFaaS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>• Channel = digital, in-person, or omnichannel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>• Proposition = what the merchant buys (e.g. Genius S, WP360, Revenue Boost). Propositions are inputs and milestones, not an axis of this view.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>• Platform = the stack itself, current vs target.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>• Persona treatment: SMB is not split by persona; Integrated tags personas inline in brackets; Enterprise is to be decided.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Open questions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>1. Which countries do we consider per region? We want to avoid the long tail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>2. Enterprise: do we split by persona / vertical (region × top 1–4 verticals)? Decide before populating further.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>3. Reconcile platform retirement timelines with the data centre consolidation plan — preliminary view requested from infrastructure (an application kept for three years cannot sit in a data centre exiting in one).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>4. North America is intentionally omitted from this June pack — it is sequenced for the Jul 20–21 in-person.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>5. All populated content is a straw man from the June QPRs and workshop discussions — validate or clear with the segment and geo leads.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Aggregate priorities (segment-wide, 2026–27):</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>• Standardization and platform unification (POM + TAM).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>• Onboarding and activation speed — the core growth bottleneck.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>• VAS monetization — lending, payments optimization, settlement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>• Execution discipline — customer commitments and large rollouts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>• Migration off legacy and reduction of fragmentation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Enterprise segment priorities:</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="70" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>• 2026 — Expand global payment capabilities (APMs, card acceptance, hosted payouts and in-app solutions). Enable complex enterprise use cases (marketplace and platform capabilities: split payments, cross-border collection, embedded payouts and treasury flows). Launch next-gen commerce (agentic commerce foundations; tokenized payments and AI integrations). Optimize partner and cost structure (third-party dependencies, partner agreements, commercial models).</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="42" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
           <t>• 2027 — Platform for global enterprise commerce (global payments, marketplaces, embedded finance). Scale next-gen commerce (card networks, AI ecosystems). Marketplace dominance at scale (split payments, cross-border collection, embedded payouts and treasury flows). Complete global APM coverage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Enterprise notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="42" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>• Persona / vertical split is an open decision — candidate structure is region × top 1–4 priority verticals (per QPR sales mix: Financial Services &amp; Healthcare, Travel &amp; Airlines, Gaming, Digital/Media). Decide before populating further.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="42" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>• Capacity trade-offs already tabled by the segment feed the stop-list: Payermax and Pix Brazil delayed (resource moved to Wero); Klarna Network US pushed ~1 PI for US Pay-by-Bank. These are sequencing decisions for the workshop, not BAU noise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>• Populated as a straw man from the June 2026 Enterprise QPR and workshop discussions — for reaction with the segment leads (Fry / Jacobs).</t>
         </is>
       </c>
     </row>
@@ -889,12 +777,18 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -912,11 +806,15 @@
 6. Partner &amp; cost structure — renegotiate agreements ($5m target), reduce third-party dependencies</t>
         </is>
       </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="17" t="n"/>
     </row>
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Corporate priorities / constraints</t>
+          <t>Corporate priorities</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -927,13 +825,23 @@
 • WP Total end-of-life — triPOS option currently points at MBoss, which is not the long-term answer; replacement must include real-time reporting or customers will leave</t>
         </is>
       </c>
-    </row>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="17" t="n"/>
+    </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -1967,12 +1875,18 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -1990,11 +1904,15 @@
 6. GMAS EU enterprise back-book — migration to NAP as the expansion unlock</t>
         </is>
       </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="17" t="n"/>
     </row>
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Corporate priorities / constraints</t>
+          <t>Corporate priorities</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2005,13 +1923,23 @@
 • Klarna Network GA RoW — migrating merchants off legacy MOR architecture onto WPG/Access</t>
         </is>
       </c>
-    </row>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="17" t="n"/>
+    </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -2989,12 +2917,18 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -3010,11 +2944,15 @@
 4. Payermax for SEA — preferred local payment methods where APMs dominate share of wallet (delayed by the Wero trade-off)</t>
         </is>
       </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="17" t="n"/>
     </row>
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Corporate priorities / constraints</t>
+          <t>Corporate priorities</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3024,13 +2962,23 @@
 • JCB tokenization spans CMP, RB, PET, WPG and NAP — multi-train coordination</t>
         </is>
       </c>
-    </row>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="17" t="n"/>
+    </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -3977,12 +3925,18 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -3995,11 +3949,15 @@
           <t>(populate ahead of June workshop)</t>
         </is>
       </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="17" t="n"/>
     </row>
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Corporate priorities / constraints</t>
+          <t>Corporate priorities</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
@@ -4007,13 +3965,23 @@
           <t>(populate ahead of June workshop)</t>
         </is>
       </c>
-    </row>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="17" t="n"/>
+    </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Replace cross-geo tabs with geo distribution incl. North America tabs
Platform view / Global tabs removed. Content re-housed by where it
serves: NA tabs (pre-seeded for Jul 20-21) carry VAP/ACH, SF.com,
Payrix, PayFac suite, Assist, EFE, agentic commerce, Pay-by-Bank US,
Interac, franchisee automation, Revenue Boost/eDCC NA items. Europe
gains WP Total exit, Genius enterprise omnichannel, marketplace
hosted payouts and seller KYB, FX/MCP+ and FraudSight items. The
segment-wide Access-only API policy is repeated per populated geo tab
and labeled as such. Workshop-pack subtitle updated to include NA.

https://claude.ai/code/session_011p8iTtbymDUbCg8RtXLgqJ
</commit_message>
<xml_diff>
--- a/TAM2.0_Sequencing_Prework_Enterprise_v0.2.xlsx
+++ b/TAM2.0_Sequencing_Prework_Enterprise_v0.2.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="How to read" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Global — cross-region" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="North America" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Europe" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="APAC" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Oceania" sheetId="5" state="visible" r:id="rId5"/>
@@ -54,6 +54,11 @@
       <sz val="13"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="9"/>
@@ -79,11 +84,6 @@
     </font>
     <font>
       <color rgb="00000000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00595959"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -115,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -137,55 +137,11 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -202,38 +158,39 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -615,11 +572,10 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>June workshop pack: Europe · APAC · Oceania</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Workshop pack: Europe · APAC · Oceania (June) · North America (Jul 20–21)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -683,7 +639,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -726,7 +681,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -773,136 +727,122 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>TAM 2.0 sequencing — Enterprise · Global — cross-region</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>TAM 2.0 sequencing — Enterprise · North America</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Pre-seeded for the Jul 20–21 North America sequencing session.</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Business priorities</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>1. Single front door — constrain new enterprise API builds to Access / the front-end API ahead of API 2.0; one API with all value-added services exposed
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>1. Pay-by-Bank US — GPPaaS completes PI2, Core (RAFT and EF) in PI3, end-to-end testing late Q3 / early Q4; Aeropay progressing on the non-guaranteed model
 2. Agentic commerce — launch 1–2 merchants on ACP/UCP; OpenAI ACP code-complete and Visa Agentic Token in certification (protocol, token and trust layers)
-3. Marketplaces — split payments, cross-border collection, seller onboarding (KYC/KYB), embedded payouts and treasury flows
-4. Omnichannel — three pillars: core card-present processing, reseller via FreedomPay, and proprietary end-to-end (Genius into QSR/FSR/Stadia in UK &amp; Europe)
-5. VAS cross-sell — FX/MCP+ and eDCC, payouts wallets (PayPal, USDC), FraudSight premier, Revenue Boost completeness
-6. Partner &amp; cost structure — renegotiate agreements ($5m target), reduce third-party dependencies</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="17" t="n"/>
+3. Interac in-app — eCom enablement for Google and Apple Pay ($19M+ Canadian pipeline)
+4. Franchisee automation — boarding API, Salesforce and Maxwell automation for Canadian merchants ($19M+ pipeline)
+5. Payouts expansion — PayPal and USDC wallets; UATP US domestic; whale-deal conversion to de-risk the payouts cross-sell gap</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Corporate priorities</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>• Pilot-readiness commitments slipping on resource constraints (OKR off-track: delays &gt;6 months)
-• Payouts cross-sell carries elevated risk — product readiness constraints; reliance on whale deals
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>• Aeropay contract unsigned; revised non-guaranteed pricing introduces material risk to the US Pay-by-Bank business case for Platforms
+• Klarna Network US pushed ~1 PI (≥Q1 '27) in favour of Pay-by-Bank — agreed trade-off
 • Revenue Boost proposition completeness — boarding and reporting limitations driving poor merchant experience
-• WP Total end-of-life — triPOS option currently points at MBoss, which is not the long-term answer; replacement must include real-time reporting or customers will leave</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="17" t="n"/>
-    </row>
-    <row r="6"/>
+• eDCC for US/CAN hospitality — did not make the PI2 cutline; sizing under way</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Workstream</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Current-state stack</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Target-state stack (validate)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Now (H2 '26 – H1 '27)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Next (H2 '27 – H1 '29)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Later (H2 '29+)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Milestones ▼</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>▼ Agentic commerce — first 1–2 merchants live on ACP/UCP
-▼ Klarna Network GA RoW</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>▼ WP Total replacement defined and in market</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr"/>
+▼ Pay-by-Bank US end-to-end testing late Q3 / early Q4 '26</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>▼ Klarna Network US ≥Q1 '27 (post trade-off)</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr"/>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Single-in</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -920,7 +860,6 @@
               <sz val="9"/>
             </rPr>
             <t>• Access Worldpay
-• WPG
 • TAPI (persists, corporate)
 • GP eCom API / GP-API (hGP)</t>
           </r>
@@ -941,12 +880,11 @@
               <sz val="9"/>
             </rPr>
             <t>• FreedomPay (reseller)
-• triPOS
-• WP Total (end-of-life path)</t>
-          </r>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
+• triPOS</t>
+          </r>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1023,32 +961,27 @@
           </r>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>• [STOP] Constrain new enterprise API builds to Access / the front-end API — single-in policy ahead of API 2.0
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>• [STOP] Constrain new enterprise API builds to Access / the front-end API — segment-wide policy ahead of API 2.0
 • [BUILD] Agentic commerce foundations — complete OpenAI ACP and Visa Agentic Token certification; launch 1–2 merchants on ACP/UCP — enabling the next-gen commerce priority</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>• [MIGRATE] Converge Access onto the API 2.0 / Global API standard (federated build to spec)
-• [BUILD] Genius into the enterprise omnichannel offer (QSR/FSR/Stadia) on the target SDK path — full end-to-end replacing the referral model</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>• [EXIT] Decommission legacy enterprise APIs once back-books converge</t>
-        </is>
-      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>• [MIGRATE] Converge Access onto the API 2.0 / Global API standard (federated build to spec)</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Boarding</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1195,27 +1128,26 @@
           </r>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] Unified franchisee platform and automation — automated onboarding, compliance and POS rental replacing custom-built setups
-• [BUILD] Marketplace seller onboarding (KYC/KYB) — fold into the pan-TAM KYB/KYC approach and partner selection</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Unified franchisee platform and automation — boarding API, Salesforce and Maxwell automation for Canadian merchants, replacing custom-built setups</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>• [BUILD] Auto-boarding end to end across gateway systems down to APM partners — supporting payfac and marketplace setups at scale</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
     </row>
     <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Servicing</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1272,17 +1204,17 @@
           </r>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Payment Processing</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1299,14 +1231,13 @@
               <color rgb="002F5496"/>
               <sz val="9"/>
             </rPr>
-            <t>• VAP
+            <t>• VAP — NA only
 • Core
-• GMAS estates (hGP)
-• NAP (target back end)</t>
-          </r>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
+• RAFT</t>
+          </r>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1401,30 +1332,27 @@
           </r>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] Hosted payouts marketplace launch — fully hosted payouts distribution, reducing integration friction for marketplaces</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>• [MIGRATE] WP Total exit — define the proprietary triPOS-based replacement (MBoss pointing is tactical at best); must carry real-time reporting to avoid attrition
-• [BUILD] Payouts expansion — PayPal and USDC wallets, UATP US domestic</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>• [EXIT] Decommission WP Total</t>
-        </is>
-      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Pay-by-Bank US — GPPaaS, Core (RAFT/EF) and end-to-end testing; low-code integration model removing APM adoption friction
+• [BUILD] Interac in-app enablement (ETP, ~1 PI) — unlocking top Canadian opportunities</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Klarna Network US (re-sequenced ≥Q1 '27 after the Pay-by-Bank trade-off)
+• [BUILD] Payouts expansion — PayPal and USDC wallets; UATP US domestic</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr"/>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>VAS</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1442,13 +1370,12 @@
               <sz val="9"/>
             </rPr>
             <t>• Revenue Boost
-• FraudSight/Ravelin
-• MCP / FX
+• FraudSight / Ravelin
 • Separate authentication &amp; routing services (sold separately today)</t>
           </r>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1595,28 +1522,28 @@
           </r>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] FraudSight premier UI enablement; Ravelin integration to both hWP and hGP gateways — one fraud answer either side of the estate
-• [BUILD] Revenue Boost completeness — integrated debit routing and intelligent token decisioning
-• [BUILD] FX — eDCC widening and live FX (&lt;10-minute onboarding), extending the MCP+ moat</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] Bring optimization and authentication services under the single intelligent decision layer — sold as a suite, not separate products</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Revenue Boost completeness — integrated debit routing and intelligent token decisioning
+• [BUILD] FraudSight premier UI enablement; Ravelin integration to both hWP and hGP gateways — one fraud answer either side of the estate</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Bring optimization and authentication services under the single intelligent decision layer — sold as a suite, not separate products
+• [BUILD] eDCC for US/CAN hospitality (sizing in progress)</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr"/>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Unified Data and AI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1655,18 +1582,18 @@
           </r>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Global Infrastructure &amp; Security (incl. data centres)</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1741,18 +1668,18 @@
           </r>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Single-out</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1827,21 +1754,14 @@
           </r>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] Hosted payouts directly in the portal — removes merchant dev-prioritisation dependency (UKVI, Disney, Next, Qatar Airways; ~$1M plus product pull-through)</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] Payout rules and reconciliation reporting — closing the proposition gap that limits marketplace scalability</t>
-        </is>
-      </c>
-      <c r="F17" s="14" t="inlineStr"/>
+      <c r="D17" s="15" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A3:F3"/>
@@ -1875,134 +1795,159 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Business priorities</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>1. Wero — start build in PI3 (GPP, Plutus and WPAP trains) to protect iDEAL revenue (~$1.7m p.a.) and top-tier merchants (Disney, Apple, Etsy, Bet365) ahead of iDEAL decommissioning Q4 '27; merchants need 8–12 months to integrate
 2. Marketplaces — APM enablement for split payments across ~60% of EU countries (Germany, Poland, Netherlands, Nordics, Italy, Belgium ≈ 50% of EU eCom GMV); $9.3M lost to date, $14M+ active pipeline
 3. Jaywan enablement — mandated in the UAE; Q3 go-live dependent on credential management and MPLS connectivity
 4. Vipps/MobilePay for the Nordics — required for the ~$1m Miinto deal
 5. Reach — global Merchant-of-Record enablement (Tier-1 interest incl. META)
-6. GMAS EU enterprise back-book — migration to NAP as the expansion unlock</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="17" t="n"/>
+6. Omnichannel — Genius into enterprise QSR/FSR/Stadia for UK &amp; Europe; WP Total replacement
+7. GMAS EU enterprise back-book — migration to NAP as the expansion unlock</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Corporate priorities</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>• iDEAL decommissioning Q4 '27 — hard external date; Wero capacity not available across APM trains in PI3/PI4 without trade-offs (Payermax and Pix delayed to fund it)
+• WP Total end-of-life — the triPOS option currently points at MBoss, which is not the long-term answer; replacement must carry real-time reporting or customers will leave
 • Jaywan — lack of clarity from the credential management team on timelines (escalated)
 • GMAS EU / FIS separation — migration waves 2028 (corporate)
-• Klarna Network GA RoW — migrating merchants off legacy MOR architecture onto WPG/Access</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="17" t="n"/>
-    </row>
-    <row r="6"/>
+• FX — eDCC widening and live FX (&lt;10-minute onboarding) extend the MCP+ moat for the airline-heavy book</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Workstream</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Current-state stack</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Target-state stack (validate)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Now (H2 '26 – H1 '27)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Next (H2 '27 – H1 '29)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Later (H2 '29+)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Milestones ▼</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>▼ Jaywan go-live Q3 '26 (UAE mandate)
-▼ Wero build starts PI3</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
+▼ Wero build starts PI3
+▼ Klarna Network GA RoW</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>▼ iDEAL decommissioning Q4 '27 (Wero integrated 8–12 months prior)
+▼ WP Total replacement defined and in market
 ▼ GMAS EU / FIS migration waves 2028</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr"/>
+      <c r="F9" s="13" t="inlineStr"/>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Single-in</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr"/>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">Front doors
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• Access Worldpay
+• WPG</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+Card present
+</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="002F5496"/>
+              <sz val="9"/>
+            </rPr>
+            <t>• WP Total (end-of-life path)
+• FreedomPay (reseller)
+• Genius (referral today)</t>
+          </r>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2079,22 +2024,28 @@
           </r>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] Reach — global Merchant-of-Record enablement via Access and WPG (Tier-1 interest incl. META)</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>• [STOP] Constrain new enterprise API builds to Access / the front-end API — segment-wide policy ahead of API 2.0
+• [BUILD] Reach — global Merchant-of-Record enablement via Access and WPG (Tier-1 interest incl. META)</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>• [MIGRATE] Converge Access onto the API 2.0 / Global API standard (federated build to spec)
+• [BUILD] Genius into the enterprise omnichannel offer (QSR/FSR/Stadia, UK &amp; Europe) on the target SDK path — full end-to-end replacing the referral model</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Boarding</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2241,18 +2192,22 @@
           </r>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Marketplace seller onboarding (KYC/KYB) — fold into the pan-TAM KYB/KYC approach and partner selection</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
     </row>
     <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Servicing</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2309,17 +2264,17 @@
           </r>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Payment Processing</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2361,7 +2316,7 @@
           </r>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2456,35 +2411,38 @@
           </r>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>• [BUILD] Wero — start build PI3 across GPP/Plutus/WPAP — protecting iDEAL-dependent revenue and top-tier merchants
 • [BUILD] Jaywan enablement (3 teams; credential management dependency) — mandated in the UAE
 • [BUILD] Vipps/MobilePay for the Nordics — enabling the Miinto deal and Nordic TAM
-• [BUILD] Marketplace APM enablement for split payments (WPG + MPM) — enabling the marketplace addressability priority (14% → 40%)</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
+• [BUILD] Marketplace APM enablement for split payments (WPG + MPM) — enabling the marketplace addressability priority (14% → 40%)
+• [BUILD] Hosted Payouts marketplace solution — fully hosted payouts distribution, reducing integration friction</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>• [EXIT] iDEAL decommissioning Q4 '27 (post-Wero migration)
 • [MIGRATE] Klarna RoW merchants off legacy MOR architecture onto WPG/Access
-• [MIGRATE] GMAS EU enterprise back-book → NAP (FIS waves 2028) — new locations and products then route via converged rails</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>• [EXIT] Complete the GMAS EU exit</t>
+• [MIGRATE] GMAS EU enterprise back-book → NAP (FIS waves 2028) — new locations and products then route via converged rails
+• [MIGRATE] WP Total exit — define the proprietary triPOS-based replacement (MBoss pointing is tactical at best)</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>• [EXIT] Complete the GMAS EU exit
+• [EXIT] Decommission WP Total</t>
         </is>
       </c>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>VAS</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr"/>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2631,18 +2589,23 @@
           </r>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] FX — eDCC widening and live FX (&lt;10-minute onboarding), extending the MCP+ moat
+• [BUILD] FraudSight premier — UI enablement and the gambling SAM campaign</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr"/>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Unified Data and AI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2681,18 +2644,18 @@
           </r>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Global Infrastructure &amp; Security (incl. data centres)</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2767,17 +2730,17 @@
           </r>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Single-out</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2798,7 +2761,7 @@
           </r>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2873,13 +2836,17 @@
           </r>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>• [BUILD] Hosted payouts in the portal (1 team, 1 PI) — UKVI, Disney, Next, Qatar Airways</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Hosted payouts directly in the portal (1 team, 1 PI) — removes merchant dev-prioritisation dependency (UKVI, Disney, Next, Qatar Airways; ~$1M plus product pull-through)</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>• [BUILD] Payout rules and reconciliation reporting — closing the proposition gap that limits marketplace scalability</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2917,26 +2884,20 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Business priorities</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>1. Japan — JCB proxy aggregator launch (B2B + PayFac acceptance of Japan's second-largest network without a direct relationship); JCB network tokenization next (auth-rate uplift, reduced proxy fees)
 2. Alipay+ scale-out — single connection unlocking 17 dominant APMs; live with Garuda, Lensemode, NEXT
@@ -2944,104 +2905,90 @@
 4. Payermax for SEA — preferred local payment methods where APMs dominate share of wallet (delayed by the Wero trade-off)</t>
         </is>
       </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="17" t="n"/>
     </row>
     <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Corporate priorities</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>• Taiwan data localisation — current stack is not cloud-ready in-market; fundamental TAM work required before a CyberSource replacement can be offered
 • Payermax delivery pushed from Q4 '26 to ≥Q1 '27 (capacity moved to Wero); $8.3M p.a. acquiring ACV at risk plus $1.8M pipeline
 • JCB tokenization spans CMP, RB, PET, WPG and NAP — multi-train coordination</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="17" t="n"/>
-    </row>
-    <row r="6"/>
+    </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Workstream</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Current-state stack</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Target-state stack (validate)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Now (H2 '26 – H1 '27)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Next (H2 '27 – H1 '29)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Later (H2 '29+)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Milestones ▼</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>▼ Japan JCB proxy aggregator launch Q3 '26
 ▼ Alipay+ live (17 APMs)</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>▼ CyberSource Taiwan connection end-of-life '27
 ▼ Payermax delivery ≥Q1 '27 (post-trade-off)</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr"/>
+      <c r="F9" s="13" t="inlineStr"/>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Single-in</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr"/>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr"/>
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3118,22 +3065,26 @@
           </r>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>• [STOP] Constrain new enterprise API builds to Access / the front-end API — segment-wide policy ahead of API 2.0</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>• [BUILD] Card-present solution and certification for APAC enterprise — required before hGP CP back-books (omnichannel, hotels) can move to target rails</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr"/>
+      <c r="F10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Boarding</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3280,18 +3231,18 @@
           </r>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
     </row>
     <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Servicing</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3348,17 +3299,17 @@
           </r>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Payment Processing</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3399,7 +3350,7 @@
           </r>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3494,29 +3445,29 @@
           </r>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>• [BUILD] Japan JCB proxy aggregator — acceptance without a direct relationship, expanding the addressable footprint
 • [BUILD] Scale Alipay+ — 17 APMs through one connection, enabling the geo-presence priority</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>• [BUILD] Taiwan data-localisation path — cloud-ready stack to replace the end-of-life CyberSource connection and retain Tier-1s (Apple)
 • [BUILD] JCB network tokenization across CMP/RB/PET/WPG/NAP — auth-rate uplift and reduced Japan proxy fees
 • [BUILD] Payermax for SEA (re-sequenced ≥Q1 '27 after the Wero trade-off)</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr"/>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>VAS</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr"/>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3663,18 +3614,18 @@
           </r>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr"/>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Unified Data and AI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3713,18 +3664,18 @@
           </r>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Global Infrastructure &amp; Security (incl. data centres)</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3799,18 +3750,18 @@
           </r>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Single-out</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3885,9 +3836,9 @@
           </r>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr"/>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
+      <c r="D17" s="15" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3925,116 +3876,96 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4" ht="62" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Business priorities</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>(populate ahead of June workshop)</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="17" t="n"/>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>(populate ahead of the workshop)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Corporate priorities</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>(populate ahead of June workshop)</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="17" t="n"/>
-    </row>
-    <row r="6"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>(populate ahead of the workshop)</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>SEQUENCING</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Workstream</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Current-state stack</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Target-state stack (validate)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Now (H2 '26 – H1 '27)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Next (H2 '27 – H1 '29)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Later (H2 '29+)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Milestones ▼</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="12" t="inlineStr"/>
-      <c r="F9" s="12" t="inlineStr"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="13" t="inlineStr"/>
+      <c r="E9" s="13" t="inlineStr"/>
+      <c r="F9" s="13" t="inlineStr"/>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Single-in</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr"/>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr"/>
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4111,18 +4042,18 @@
           </r>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
+      <c r="D10" s="15" t="inlineStr"/>
+      <c r="E10" s="15" t="inlineStr"/>
+      <c r="F10" s="15" t="inlineStr"/>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Boarding</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4269,18 +4200,18 @@
           </r>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
     </row>
     <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Sales &amp; Servicing</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4337,18 +4268,18 @@
           </r>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Payment Processing</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr"/>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr"/>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4443,18 +4374,18 @@
           </r>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
+      <c r="D13" s="15" t="inlineStr"/>
+      <c r="E13" s="15" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr"/>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>VAS</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr"/>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4601,18 +4532,18 @@
           </r>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr"/>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Unified Data and AI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4651,18 +4582,18 @@
           </r>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
+      <c r="D15" s="15" t="inlineStr"/>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Global Infrastructure &amp; Security (incl. data centres)</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4737,18 +4668,18 @@
           </r>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Single-out</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4823,9 +4754,9 @@
           </r>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr"/>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
+      <c r="D17" s="15" t="inlineStr"/>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>